<commit_message>
upload folloing final modelling
</commit_message>
<xml_diff>
--- a/tools/spatial_prob_manipulations_details.xlsx
+++ b/tools/spatial_prob_manipulations_details.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20398"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26626"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\CH_ValPar.CH\03_workspaces\07_Modeling\LULCC_CH\Tools\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bblack\switchdrive\C.3_Modelling\LULCC_CH\Tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93A30DE0-4E83-4AC7-9EFC-09A35DD4D870}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B8F5CA5-13DD-4047-9E29-0A617B0A58EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12225" xr2:uid="{651BAE16-29FB-4958-8697-D574B39FF50C}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10395" xr2:uid="{651BAE16-29FB-4958-8697-D574B39FF50C}"/>
   </bookViews>
   <sheets>
     <sheet name="Spatial_prob_perturb_suggestion" sheetId="1" r:id="rId1"/>
@@ -42,148 +42,76 @@
   <commentList>
     <comment ref="I13" authorId="0" shapeId="0" xr:uid="{6F01B808-00D3-49DE-92E6-02799E50627C}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t xml:space="preserve">[Threaded comment]
+        <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     What is again the logic of a rural exodus in the BAU scenario?
 Reply:
     Because in the BAU I also see the devlopment with all the holiday houses to continue.  </t>
-        </r>
       </text>
     </comment>
     <comment ref="I14" authorId="1" shapeId="0" xr:uid="{402ED776-0F76-4DD4-AABA-DA4B3D344E82}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t xml:space="preserve">[Threaded comment]
+        <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     What is again the logic of a rural exodus in the BAU scenario?
 Reply:
     Because in the BAU I also see the devlopment with all the holiday houses to continue.  </t>
-        </r>
       </text>
     </comment>
     <comment ref="I15" authorId="2" shapeId="0" xr:uid="{D8018EB7-F89F-E54B-B0CE-75895A5D894E}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t xml:space="preserve">[Threaded comment]
+        <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     What is again the logic of a rural exodus in the BAU scenario?
 Reply:
     Because in the BAU I also see the devlopment with all the holiday houses to continue.  </t>
-        </r>
       </text>
     </comment>
     <comment ref="I17" authorId="3" shapeId="0" xr:uid="{49FAC4C3-F42B-4A16-B5FA-FB831116C489}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t xml:space="preserve">[Threaded comment]
+        <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     What is again the logic of a rural exodus in the BAU scenario?
 Reply:
     Because in the BAU I also see the devlopment with all the holiday houses to continue.  </t>
-        </r>
       </text>
     </comment>
     <comment ref="I18" authorId="4" shapeId="0" xr:uid="{645B1E99-411A-4ECC-B3F9-0789F2C90FE5}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t xml:space="preserve">[Threaded comment]
+        <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     What is again the logic of a rural exodus in the BAU scenario?
 Reply:
     Because in the BAU I also see the devlopment with all the holiday houses to continue.  </t>
-        </r>
       </text>
     </comment>
     <comment ref="H19" authorId="5" shapeId="0" xr:uid="{DC6CB4E6-37EC-FC48-9A5E-04ECF2D274DF}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t xml:space="preserve">[Threaded comment]
+        <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Here I think it’s a question of time when this land starts to shift to another class which likely is shrubland or forest. Depending on how long these processes take. </t>
-        </r>
       </text>
     </comment>
     <comment ref="H20" authorId="6" shapeId="0" xr:uid="{309C492E-E860-43C2-B03F-4829E925F5CC}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t xml:space="preserve">[Threaded comment]
+        <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Here I think it’s a question of time when this land starts to shift to another class which likely is shrubland or forest. Depending on how long these processes take. </t>
-        </r>
       </text>
     </comment>
     <comment ref="H21" authorId="7" shapeId="0" xr:uid="{2BC2C279-6A71-4933-9130-A7B8727E337D}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t xml:space="preserve">[Threaded comment]
+        <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Here I think it’s a question of time when this land starts to shift to another class which likely is shrubland or forest. Depending on how long these processes take. </t>
-        </r>
       </text>
     </comment>
   </commentList>
@@ -191,7 +119,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="86">
   <si>
     <t>Scenario</t>
   </si>
@@ -247,9 +175,6 @@
     <t>Intervention_ID</t>
   </si>
   <si>
-    <t>probability of Urban transitions increased inside building zones (using all classes in the building zones)</t>
-  </si>
-  <si>
     <t>alter values of allocation parameter (patcher vs. Expander)</t>
   </si>
   <si>
@@ -298,12 +223,6 @@
     <t>Mountain_development</t>
   </si>
   <si>
-    <t>Use Typology of municipalities with 25 categories to identify cells and increase probability to urban</t>
-  </si>
-  <si>
-    <t>Use Typology of municipalities with 25 categories to identify cells and decrease probability to urban</t>
-  </si>
-  <si>
     <t>Data/Spat_prob_perturb_layers/Municipality_typology/Muni_type_raster.grd</t>
   </si>
   <si>
@@ -337,28 +256,16 @@
     <t>Mechanism_detailed</t>
   </si>
   <si>
-    <t>Alter values of allocation parameters : Increase % of transitions with expander (incurring decrease in patcher %)</t>
-  </si>
-  <si>
     <t>spatial_zoning</t>
   </si>
   <si>
     <t>Increase in probability of transition of marginal agricultural land to non-agricultural classes</t>
   </si>
   <si>
-    <t>decrease in probability of marginal agricultural land transitioning to other classes</t>
-  </si>
-  <si>
     <t>Alp_Past</t>
   </si>
   <si>
     <t xml:space="preserve"> Alp_Past</t>
-  </si>
-  <si>
-    <t>Identify marginal agricultural land using an index (0-1) of slope, distance to roads, inverse distance to building zones and elevation (Müller 2022). Select 90th percentile of most marginal pixels and then select 95th percentile of pixels according to probability and decrease  probability to transition from Agriculture by 5%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Identify marginal agricultural land using an index (0-1) of slope, distance to roads, inverse distance to building zones and elevation (Müller 2022). Select upper quartile of most marginal pixels and then select 90th percentile of pixels according to probability and  increase probability to transition from Agriculture to non-agricultural classes. Simultaneously select pixels below upper quartile of marginality and then select 90th percentile of pixels according to probability and  decrease probability to transition from Agriculture to non-agricultural classes. </t>
   </si>
   <si>
     <t>N</t>
@@ -435,7 +342,43 @@
     <t>"Extensive cultivation of poorly accessible marginal land"</t>
   </si>
   <si>
-    <t>Spatial prioritization map produced with the conservation prioritization software Zonation [@lehtomäki2013] using modelled spatial data for 7 NCPs: nutrient retention; recreation; landscape suitability for pollination; pest control; hazard regulation; carbon storage in vegetation; air quality regulation.</t>
+    <t>Increase % of transitions with expander (incurring decrease in patcher %)</t>
+  </si>
+  <si>
+    <t>Increase probability to urban of cells in Mountainous municipalities</t>
+  </si>
+  <si>
+    <t>Decrease probability to urban of cells in remote rural municipalities</t>
+  </si>
+  <si>
+    <t>Increase probability to urban of cells in remote rural municipalities</t>
+  </si>
+  <si>
+    <t>Decrease in probability of marginal agricultural land transitioning to other classes</t>
+  </si>
+  <si>
+    <t>Select 90th percentile of most marginal pixels and then select 95th percentile of pixels according to probability and decrease  probability to transition from Agriculture by 5%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Select upper quartile of most marginal pixels and then select 90th percentile of pixels according to probability and  increase probability to transition from Agriculture to non-agricultural classes. Simultaneously select pixels below upper quartile of marginality and then select 90th percentile of pixels according to probability and  decrease probability to transition from Agriculture to non-agricultural classes. </t>
+  </si>
+  <si>
+    <t>Probability of Urban transitions increased inside building zones (using all classes in the building zones)</t>
+  </si>
+  <si>
+    <t>Marginal agricultural land identified using an index (0-1) of slope, distance to roads, inverse distance to building zones and elevation[@muller_verbuschung_2022].</t>
+  </si>
+  <si>
+    <t>Areas to modify urban development identified using the Swiss building zones geodata \citepalias{ARE_2022}.</t>
+  </si>
+  <si>
+    <t>Mountainous municipalities identified using the Swiss typology of municipalities (25 categories)\citepalias{swiss_federal_office_for_statistics_sfso_typology_2023}</t>
+  </si>
+  <si>
+    <t>For details see @sec-PA_process</t>
+  </si>
+  <si>
+    <t>Remote rural municipalities identified using the Swiss typology of municipalities (25 categories)\citepalias{swiss_federal_office_for_statistics_sfso_typology_2023}</t>
   </si>
 </sst>
 </file>
@@ -1038,22 +981,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8ACA9C24-578D-43A9-82B8-6427B2AE2C72}">
   <dimension ref="A1:K25"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="25.42578125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="15.42578125" style="1" hidden="1" customWidth="1"/>
-    <col min="3" max="4" width="52.5703125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="29.42578125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="17.42578125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="25.42578125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="25.3984375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="15.3984375" style="1" hidden="1" customWidth="1"/>
+    <col min="3" max="4" width="52.59765625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="29.3984375" style="1" customWidth="1"/>
+    <col min="6" max="6" width="17.3984375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="25.3984375" style="1" customWidth="1"/>
     <col min="8" max="8" width="43" style="1" customWidth="1"/>
-    <col min="9" max="9" width="59.5703125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="73.7109375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="59.59765625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="73.73046875" style="1" customWidth="1"/>
     <col min="11" max="11" width="19" style="1" customWidth="1"/>
-    <col min="12" max="16384" width="8.85546875" style="1"/>
+    <col min="12" max="16384" width="8.86328125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1061,13 +1004,13 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>2</v>
@@ -1076,19 +1019,19 @@
         <v>17</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="71.25" x14ac:dyDescent="0.45">
       <c r="A2" s="4" t="s">
         <v>3</v>
       </c>
@@ -1096,34 +1039,34 @@
         <v>4</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>48</v>
+        <v>73</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="K2" s="17" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A3" s="4" t="s">
         <v>6</v>
       </c>
@@ -1131,34 +1074,34 @@
         <v>4</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>48</v>
+        <v>73</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="K3" s="17" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="96" customHeight="1" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="96" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="23" t="s">
         <v>7</v>
       </c>
@@ -1166,19 +1109,19 @@
         <v>8</v>
       </c>
       <c r="C4" s="24" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="D4" s="24" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="E4" s="23" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F4" s="23" t="s">
         <v>9</v>
       </c>
       <c r="G4" s="23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H4" s="23" t="s">
         <v>10</v>
@@ -1187,13 +1130,13 @@
         <v>10</v>
       </c>
       <c r="J4" s="23" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="K4" s="25" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="122.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="122.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="23" t="s">
         <v>11</v>
       </c>
@@ -1201,19 +1144,19 @@
         <v>8</v>
       </c>
       <c r="C5" s="24" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="D5" s="24" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F5" s="23" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="G5" s="23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H5" s="23" t="s">
         <v>10</v>
@@ -1222,13 +1165,13 @@
         <v>10</v>
       </c>
       <c r="J5" s="25" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="K5" s="25" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="68.849999999999994" customHeight="1" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="68.849999999999994" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="23" t="s">
         <v>3</v>
       </c>
@@ -1236,34 +1179,34 @@
         <v>8</v>
       </c>
       <c r="C6" s="24" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="D6" s="24" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F6" s="23" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="G6" s="23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H6" s="23" t="s">
         <v>10</v>
       </c>
       <c r="I6" s="32" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="J6" s="33" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="K6" s="25" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" ht="105" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="85.5" x14ac:dyDescent="0.45">
       <c r="A7" s="23" t="s">
         <v>12</v>
       </c>
@@ -1271,32 +1214,34 @@
         <v>8</v>
       </c>
       <c r="C7" s="24" t="s">
-        <v>70</v>
-      </c>
-      <c r="D7" s="24"/>
+        <v>63</v>
+      </c>
+      <c r="D7" s="24" t="s">
+        <v>84</v>
+      </c>
       <c r="E7" s="23" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F7" s="23" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="G7" s="23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H7" s="23" t="s">
         <v>10</v>
       </c>
       <c r="I7" s="23" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="J7" s="33" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="K7" s="25" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="46.5" x14ac:dyDescent="0.45">
       <c r="A8" s="23" t="s">
         <v>6</v>
       </c>
@@ -1304,32 +1249,34 @@
         <v>8</v>
       </c>
       <c r="C8" s="24" t="s">
-        <v>71</v>
-      </c>
-      <c r="D8" s="24"/>
+        <v>64</v>
+      </c>
+      <c r="D8" s="24" t="s">
+        <v>84</v>
+      </c>
       <c r="E8" s="23" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F8" s="23" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="G8" s="23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H8" s="23" t="s">
         <v>10</v>
       </c>
       <c r="I8" s="32" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="J8" s="33" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="K8" s="25" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A9" s="5" t="s">
         <v>12</v>
       </c>
@@ -1337,32 +1284,34 @@
         <v>13</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="D9" s="5"/>
+        <v>65</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>82</v>
+      </c>
       <c r="E9" s="6" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F9" s="5" t="s">
         <v>5</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>18</v>
+        <v>80</v>
       </c>
       <c r="I9" s="5" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="J9" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="K9" s="6" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A10" s="5" t="s">
         <v>6</v>
       </c>
@@ -1370,32 +1319,34 @@
         <v>13</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="D10" s="5"/>
+        <v>66</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>82</v>
+      </c>
       <c r="E10" s="6" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F10" s="5" t="s">
         <v>5</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>18</v>
+        <v>80</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A11" s="5" t="s">
         <v>3</v>
       </c>
@@ -1403,32 +1354,34 @@
         <v>13</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="D11" s="5"/>
+        <v>66</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>82</v>
+      </c>
       <c r="E11" s="6" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F11" s="5" t="s">
         <v>5</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>18</v>
+        <v>80</v>
       </c>
       <c r="I11" s="5" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="K11" s="6" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="85.5" x14ac:dyDescent="0.45">
       <c r="A12" s="13" t="s">
         <v>7</v>
       </c>
@@ -1436,32 +1389,34 @@
         <v>13</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>74</v>
-      </c>
-      <c r="D12" s="14"/>
+        <v>67</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>82</v>
+      </c>
       <c r="E12" s="18" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F12" s="13" t="s">
         <v>5</v>
       </c>
       <c r="G12" s="13" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H12" s="13" t="s">
         <v>14</v>
       </c>
       <c r="I12" s="13" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="J12" s="13" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="K12" s="18" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" ht="120" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="99.75" x14ac:dyDescent="0.45">
       <c r="A13" s="15" t="s">
         <v>6</v>
       </c>
@@ -1469,9 +1424,11 @@
         <v>13</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>75</v>
-      </c>
-      <c r="D13" s="15"/>
+        <v>68</v>
+      </c>
+      <c r="D13" s="15" t="s">
+        <v>83</v>
+      </c>
       <c r="E13" s="15">
         <v>314</v>
       </c>
@@ -1479,22 +1436,22 @@
         <v>5</v>
       </c>
       <c r="G13" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="H13" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="I13" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="J13" s="28" t="s">
         <v>34</v>
       </c>
-      <c r="H13" s="15" t="s">
-        <v>35</v>
-      </c>
-      <c r="I13" s="15" t="s">
-        <v>44</v>
-      </c>
-      <c r="J13" s="28" t="s">
-        <v>37</v>
-      </c>
       <c r="K13" s="19" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" ht="120" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="99.75" x14ac:dyDescent="0.45">
       <c r="A14" s="15" t="s">
         <v>3</v>
       </c>
@@ -1502,9 +1459,11 @@
         <v>13</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>75</v>
-      </c>
-      <c r="D14" s="15"/>
+        <v>68</v>
+      </c>
+      <c r="D14" s="15" t="s">
+        <v>83</v>
+      </c>
       <c r="E14" s="31">
         <v>314334</v>
       </c>
@@ -1512,22 +1471,22 @@
         <v>5</v>
       </c>
       <c r="G14" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="H14" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="I14" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="J14" s="28" t="s">
         <v>34</v>
       </c>
-      <c r="H14" s="15" t="s">
-        <v>35</v>
-      </c>
-      <c r="I14" s="15" t="s">
-        <v>44</v>
-      </c>
-      <c r="J14" s="28" t="s">
-        <v>37</v>
-      </c>
       <c r="K14" s="19" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" ht="120" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="99.75" x14ac:dyDescent="0.45">
       <c r="A15" s="7" t="s">
         <v>11</v>
       </c>
@@ -1535,32 +1494,34 @@
         <v>13</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="D15" s="8"/>
+        <v>69</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>85</v>
+      </c>
       <c r="E15" s="7" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="F15" s="7" t="s">
         <v>5</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>36</v>
+        <v>75</v>
       </c>
       <c r="I15" s="7" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="J15" s="29" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="K15" s="20" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" ht="120" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="99.75" x14ac:dyDescent="0.45">
       <c r="A16" s="7" t="s">
         <v>6</v>
       </c>
@@ -1568,32 +1529,34 @@
         <v>13</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="D16" s="7"/>
+        <v>69</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>85</v>
+      </c>
       <c r="E16" s="7" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="F16" s="7" t="s">
         <v>5</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>36</v>
+        <v>75</v>
       </c>
       <c r="I16" s="7" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="J16" s="29" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="K16" s="20" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" ht="120" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="99.75" x14ac:dyDescent="0.45">
       <c r="A17" s="7" t="s">
         <v>3</v>
       </c>
@@ -1601,32 +1564,34 @@
         <v>13</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="D17" s="7"/>
+        <v>69</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>85</v>
+      </c>
       <c r="E17" s="7" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="F17" s="7" t="s">
         <v>5</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>36</v>
+        <v>75</v>
       </c>
       <c r="I17" s="7" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="J17" s="29" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="K17" s="20" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" ht="120" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="99.75" x14ac:dyDescent="0.45">
       <c r="A18" s="26" t="s">
         <v>12</v>
       </c>
@@ -1634,32 +1599,34 @@
         <v>13</v>
       </c>
       <c r="C18" s="26" t="s">
-        <v>77</v>
-      </c>
-      <c r="D18" s="26"/>
+        <v>70</v>
+      </c>
+      <c r="D18" s="26" t="s">
+        <v>85</v>
+      </c>
       <c r="E18" s="26" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="F18" s="26" t="s">
         <v>5</v>
       </c>
       <c r="G18" s="26" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H18" s="26" t="s">
-        <v>35</v>
+        <v>76</v>
       </c>
       <c r="I18" s="26" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="J18" s="30" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="K18" s="27" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" ht="150" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="85.5" x14ac:dyDescent="0.45">
       <c r="A19" s="9" t="s">
         <v>3</v>
       </c>
@@ -1667,32 +1634,34 @@
         <v>15</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="D19" s="10"/>
+        <v>71</v>
+      </c>
+      <c r="D19" s="10" t="s">
+        <v>81</v>
+      </c>
       <c r="E19" s="9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F19" s="9" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="G19" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H19" s="9" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="I19" s="9" t="s">
-        <v>55</v>
+        <v>79</v>
       </c>
       <c r="J19" s="9" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="K19" s="21" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" ht="150" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="85.5" x14ac:dyDescent="0.45">
       <c r="A20" s="9" t="s">
         <v>11</v>
       </c>
@@ -1700,32 +1669,34 @@
         <v>15</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="D20" s="10"/>
+        <v>71</v>
+      </c>
+      <c r="D20" s="10" t="s">
+        <v>81</v>
+      </c>
       <c r="E20" s="9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="I20" s="9" t="s">
-        <v>55</v>
+        <v>79</v>
       </c>
       <c r="J20" s="9" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="K20" s="21" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" ht="150" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="85.5" x14ac:dyDescent="0.45">
       <c r="A21" s="9" t="s">
         <v>16</v>
       </c>
@@ -1733,32 +1704,34 @@
         <v>15</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="D21" s="10"/>
+        <v>71</v>
+      </c>
+      <c r="D21" s="10" t="s">
+        <v>81</v>
+      </c>
       <c r="E21" s="9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F21" s="9" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="G21" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H21" s="9" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="I21" s="9" t="s">
-        <v>55</v>
+        <v>79</v>
       </c>
       <c r="J21" s="9" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="K21" s="21" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A22" s="11" t="s">
         <v>12</v>
       </c>
@@ -1766,45 +1739,47 @@
         <v>15</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>79</v>
-      </c>
-      <c r="D22" s="12"/>
+        <v>72</v>
+      </c>
+      <c r="D22" s="12" t="s">
+        <v>81</v>
+      </c>
       <c r="E22" s="11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F22" s="11" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="G22" s="11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H22" s="11" t="s">
-        <v>51</v>
+        <v>77</v>
       </c>
       <c r="I22" s="11" t="s">
-        <v>54</v>
+        <v>78</v>
       </c>
       <c r="J22" s="11" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="K22" s="22" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.45">
       <c r="C23" s="16"/>
       <c r="D23" s="16"/>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.45">
       <c r="C24" s="16"/>
       <c r="D24" s="16"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.45">
       <c r="C25" s="16"/>
       <c r="D25" s="16"/>
     </row>
   </sheetData>
-  <sortState ref="A2:K25">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K25">
     <sortCondition ref="B1"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1822,15 +1797,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100EEE3694774EF754A8CC6FC6FA5E27970" ma:contentTypeVersion="13" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="d93f88a0a8255bfb930f7a727db686ad">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="1f0a4303-6c30-4be1-95b2-d3f846a6dc61" xmlns:ns4="35f94e42-e4d5-4a2a-b205-129e91914919" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="bd2b915ebf31ecc04d3ae81b403b739a" ns3:_="" ns4:_="">
     <xsd:import namespace="1f0a4303-6c30-4be1-95b2-d3f846a6dc61"/>
@@ -2053,6 +2019,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B9B5ECA8-FED0-4F9E-AF48-225E059A944A}">
   <ds:schemaRefs>
@@ -2071,14 +2046,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E75168B6-E7FC-4BE5-9F9D-42A41711F424}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8EF3CE86-C263-48A8-AB0F-CFFD6601505F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2095,4 +2062,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E75168B6-E7FC-4BE5-9F9D-42A41711F424}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>